<commit_message>
docs: add 描述/角色协同/特殊效果 columns to deck tables
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -523,7 +523,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>本工作簿每个标签页对应一类牌堆,配合《Arena规则.md》使用。</t>
+          <t>每个标签页对应一类牌堆,配合《Arena规则.md》使用。</t>
         </is>
       </c>
     </row>
@@ -540,28 +540,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 每页第 2 行是灰色斜体【示例行】——只作格式参考,正式统计时请删除或忽略。</t>
+          <t xml:space="preserve">  • 第 2 行灰色斜体是【示例行】,只作格式参考,正式统计请忽略/删除。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 黄色底的空行是【待填区】,在这里录入你的真实牌。不够用就直接往下加行。</t>
+          <t xml:space="preserve">  • 黄色底是【待填区】,在此录入真实牌;不够就往下加行。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 蓝色标题行请勿改动列名(模拟器会按列名读取)。</t>
+          <t xml:space="preserve">  • 蓝色标题行请勿改列名(引擎会按列名读取)。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 每页底部的『张数合计』会自动加总『张数』列,用来核对整副牌的规模。</t>
+          <t xml:space="preserve">  • 底部『合计』自动加总『张数/数量』列,用来核对整副牌规模。</t>
         </is>
       </c>
     </row>
@@ -571,66 +571,69 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>六个牌堆:</t>
+          <t>三个常问的列写在哪:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1) 人物        — 每位玩家 1 张;HP 档(3/5/7)、基础攻击(2/3/4)、特殊技能</t>
+          <t xml:space="preserve">  • 描述       = 每张牌的风味文字(例:名字『蘑菇』,描述『看上去有点毒的蘑菇』)。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2) 武器        — 装备后攻击值叠加;攻击值 = 骰面数</t>
+          <t xml:space="preserve">  • 角色协同   = 某牌在特定角色手里更强(例:『刺客手中额外+2 攻击』)。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3) 弹药碎片    — 集齐拼成炸弹,炸整区所有人</t>
+          <t xml:space="preserve">  • 特殊效果   = 附加功能(例:『击杀时抽 1 张食物』『使用后可再移动一次』)。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4) 物资(食物·护甲) — 食物回血、护甲反应式减伤</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5) 随机事件    — 特定轮触发,掷 d4 定影响外区(已预填 3 个示例事件)</t>
+          <t>牌数起始建议(6 人局,约 55 张物资;可按玩家数×8~10 缩放):</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  6) 隐藏身份    — 每位玩家 1 张(秘密),个人胜利线(已预填 7 个已知身份)</t>
+          <t xml:space="preserve">  • 外区每区 ≈ 9 张:武器2(弱)/食物4/护甲3</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 中心 ≈ 11 张:武器6(含强武器+3/+4)/食物3/护甲2</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>标注约定(与规则文档一致):✅ 已确认　🔧 初值待测　❓ 待定</t>
+          <t xml:space="preserve">  • 强武器只放中心;食物/护甲别过多,否则战斗打不死人、拖慢节奏。</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>数值多为初值,请以模拟/试玩结果为准调整。</t>
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>标注约定:✅ 已确认  🔧 初值待测  ❓ 待定。数值以模拟/试玩结果为准。</t>
         </is>
       </c>
     </row>
@@ -645,16 +648,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -670,25 +674,30 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>HP档(3/5/7)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>基础攻击(2/3/4)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>特殊技能</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>张数</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -705,23 +714,28 @@
           <t>示例·游侠</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>身手敏捷的边境猎手</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>可攻击相邻区域的角色</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>技能示例,数值待定</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>技能/数值待定</t>
         </is>
       </c>
     </row>
@@ -733,6 +747,7 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -742,6 +757,7 @@
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -751,6 +767,7 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -760,6 +777,7 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -769,6 +787,7 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -778,6 +797,7 @@
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -787,6 +807,7 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -796,6 +817,7 @@
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -805,6 +827,7 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -814,6 +837,7 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -823,6 +847,7 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -832,6 +857,7 @@
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -841,6 +867,7 @@
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -850,6 +877,7 @@
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -859,6 +887,7 @@
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -868,22 +897,23 @@
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="E20" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="F20" s="7">
-        <f>SUM(F3:F18)</f>
+      <c r="G20" s="7">
+        <f>SUM(G3:G18)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>技能示例(来自规则讨论):『可攻击相邻区域的角色』『一次抽多张物资牌』。HP/攻击为初值 🔧。玩家 = 1 张人物牌 + 1 张隐藏身份牌。</t>
+          <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP/攻击为初值 🔧。</t>
         </is>
       </c>
     </row>
@@ -903,16 +933,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -928,25 +961,40 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>攻击加成(+X)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>类型(装备/一次性)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>所在区域牌堆</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>角色协同</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>特殊效果</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>张数</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -963,25 +1011,40 @@
           <t>示例·猎刀</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>一把磨得发亮的短刀</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>装备</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>任意/外区</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>刺客手中额外+2</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>击杀时抽1张食物</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>攻击值叠加到基础攻击上</t>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>攻击叠加到基础攻击上</t>
         </is>
       </c>
     </row>
@@ -993,6 +1056,9 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -1002,6 +1068,9 @@
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -1011,6 +1080,9 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -1020,6 +1092,9 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -1029,6 +1104,9 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1038,6 +1116,9 @@
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1047,6 +1128,9 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1056,6 +1140,9 @@
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1065,6 +1152,9 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1074,6 +1164,9 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1083,6 +1176,9 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1092,6 +1188,9 @@
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1101,6 +1200,9 @@
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1110,6 +1212,9 @@
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1119,6 +1224,9 @@
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1128,22 +1236,25 @@
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="E20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="F20" s="7">
-        <f>SUM(F3:F18)</f>
+      <c r="I20" s="7">
+        <f>SUM(I3:I18)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>装备后:总攻击值 = 基础攻击 + 武器加成,投掷对应面数的骰子(如总攻击 8 → d8)。武器出现频率直接影响整局节奏(B),是模拟器首要调参对象。</t>
+          <t>总攻击 = 基础攻击 + 武器加成,投掷对应面数骰(如总攻击8→d8)。角色协同/特殊效果按牌自由填写。强武器建议只放中心。</t>
         </is>
       </c>
     </row>
@@ -1163,16 +1274,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1188,25 +1301,35 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>集齐需求(几片)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>炸弹伤害</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>影响范围</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>特殊效果</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>张数</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1223,23 +1346,29 @@
           <t>示例·弹药碎片</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>锈迹斑斑的金属零件</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>整个区域所有人</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>作为附加行动埋下</t>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>附加行动埋下,下一轮爆炸</t>
         </is>
       </c>
     </row>
@@ -1251,6 +1380,8 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -1260,6 +1391,8 @@
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -1269,6 +1402,8 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -1278,6 +1413,8 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -1287,6 +1424,8 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1296,6 +1435,8 @@
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1305,6 +1446,8 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1314,6 +1457,8 @@
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1323,6 +1468,8 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1332,6 +1479,8 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1341,6 +1490,8 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1350,22 +1501,24 @@
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="E16" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="F16" s="7">
-        <f>SUM(F3:F14)</f>
+      <c r="H16" s="7">
+        <f>SUM(H3:H14)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>集齐若干碎片可拼成炸弹(附加行动埋下),炸一个区域内所有选手。几片成弹、伤害、引爆时机 ❓ 待定。</t>
+          <t>集齐若干碎片可拼成炸弹(附加行动埋下,下一轮爆炸),炸整区所有人。几片成弹/伤害 🔧 待定。</t>
         </is>
       </c>
     </row>
@@ -1385,17 +1538,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1411,30 +1566,40 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>类型(食物/护甲)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>效果</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>所在区域牌堆</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>特殊效果</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>张数</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1448,31 +1613,41 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>示例·口粮</t>
+          <t>蘑菇</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>看上去有点毒的蘑菇</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>食物</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>回复 HP</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>任意</t>
         </is>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>被某角色食用无副作用</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>回血数值待定</t>
         </is>
@@ -1487,6 +1662,8 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -1497,6 +1674,8 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -1507,6 +1686,8 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -1517,6 +1698,8 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -1527,6 +1710,8 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1537,6 +1722,8 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1547,6 +1734,8 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1557,6 +1746,8 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1567,6 +1758,8 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1577,6 +1770,8 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1587,6 +1782,8 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1597,6 +1794,8 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1607,6 +1806,8 @@
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1617,22 +1818,24 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="F18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="G18" s="7">
-        <f>SUM(G3:G16)</f>
+      <c r="I18" s="7">
+        <f>SUM(I3:I16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>食物:补充 HP。护甲:被攻击时消耗以反应式减伤(不给额外行动/抽牌)。中心区物资最丰富。</t>
+          <t>食物:补充 HP。护甲:被攻击时消耗以反应式减伤(不给额外行动/抽牌)。中心物资最丰富。特殊效果列写附加功能。</t>
         </is>
       </c>
     </row>
@@ -1652,16 +1855,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1677,25 +1881,30 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>影响区域</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>效果</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>强度</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>张数</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1714,23 +1923,28 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>遮天蔽日的黄沙</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>该区所有人本回合无法移动</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>格式示例</t>
         </is>
@@ -1747,25 +1961,26 @@
           <t>变异狼群</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>目标区所有人受 2 点攻击</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="G3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
@@ -1782,25 +1997,26 @@
           <t>洪水</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>目标区所有人弃掉手上的武器牌(已装备的除外)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="G4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
@@ -1817,25 +2033,26 @@
           <t>猴群</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>抢走目标区已装备的武器</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="G5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
@@ -1849,6 +2066,7 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -1858,6 +2076,7 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1867,6 +2086,7 @@
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1876,6 +2096,7 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1885,6 +2106,7 @@
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1894,6 +2116,7 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1903,6 +2126,7 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1912,6 +2136,7 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1921,6 +2146,7 @@
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1930,6 +2156,7 @@
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1939,6 +2166,7 @@
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1948,22 +2176,23 @@
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="E19" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="F19" s="7">
-        <f>SUM(F3:F17)</f>
+      <c r="G19" s="7">
+        <f>SUM(G3:G17)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>随机事件在特定轮触发(🔧 4/6/7/9 待商榷)。触发时先掷 d4 决定受影响外区,再抽事件牌。强度/频率需用模拟器平衡。</t>
+          <t>随机事件在特定轮触发(🔧 4/6/7/9 待商榷)。触发时先掷 d4 定受影响外区,再抽事件牌。描述列写风味文字。</t>
         </is>
       </c>
     </row>
@@ -1983,14 +2212,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2006,15 +2236,20 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>胜利条件</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>联动/备注</t>
         </is>
@@ -2033,13 +2268,18 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>独来独往的幸存者</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>游戏结束时从未结盟即胜</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>格式示例</t>
         </is>
@@ -2056,15 +2296,16 @@
           <t>Myrtle</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>最先牺牲(第一个被淘汰)即胜</t>
         </is>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="E3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -2077,15 +2318,16 @@
           <t>Social Butterfly</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>游戏结束时正确认出特殊角色(Lover/Vendetta/Bodyguard)即胜</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="E4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>需推理身份</t>
         </is>
@@ -2102,15 +2344,16 @@
           <t>Lover(爱人)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>爱上左边的玩家;若左边玩家获胜,爱人也胜</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="E5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>左右靠抽号决定</t>
         </is>
@@ -2127,15 +2370,16 @@
           <t>Sour Lemon</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>认出并杀死一名 Lover 即胜</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="E6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>与 Lover 联动</t>
         </is>
@@ -2152,15 +2396,16 @@
           <t>Warrior</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>杀敌数最多即胜</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="E7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -2173,15 +2418,16 @@
           <t>Bodyguard</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>保护 Vendetta 的复仇对象,使其不被杀</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="E8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>与 Vendetta 联动</t>
         </is>
@@ -2198,15 +2444,16 @@
           <t>Vendetta</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>杀死右边的玩家才胜(唯一条件)</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="E9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>左右靠抽号决定</t>
         </is>
@@ -2218,6 +2465,7 @@
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -2225,6 +2473,7 @@
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -2232,6 +2481,7 @@
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -2239,6 +2489,7 @@
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -2246,6 +2497,7 @@
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -2253,6 +2505,7 @@
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -2260,6 +2513,7 @@
       <c r="C16" s="5" t="n"/>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -2267,6 +2521,7 @@
       <c r="C17" s="5" t="n"/>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -2274,6 +2529,7 @@
       <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -2281,22 +2537,23 @@
       <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>张数合计</t>
-        </is>
-      </c>
-      <c r="D21" s="7">
-        <f>SUM(D3:D19)</f>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>数量合计</t>
+        </is>
+      </c>
+      <c r="E21" s="7">
+        <f>SUM(E3:E19)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>每位玩家秘密持有 1 张。允许多位胜者:每人对照自己的身份各自结算。完整清单与各身份数量 ❓ 待补。</t>
+          <t>每位玩家秘密持有 1 张。允许多位胜者:各自对照身份结算。描述列写风味文字;完整清单/数量 ❓ 待补。</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2561,7 @@
     <row r="25"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A23:E25"/>
+    <mergeCell ref="A23:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: import 10 hidden identities from Numbers, apply agreed rulings, add Judas proposal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -126,6 +126,9 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -134,9 +137,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -740,9 +740,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Growing up in a poor neighbourhood, you found ways to fit into the shadow and feed yourself without other’s noticeable.</t>
+        </is>
+      </c>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
@@ -750,7 +758,11 @@
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
@@ -760,7 +772,11 @@
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
@@ -770,7 +786,11 @@
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
@@ -780,7 +800,11 @@
       <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
@@ -790,7 +814,11 @@
       <c r="H7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
@@ -800,7 +828,11 @@
       <c r="H8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
@@ -810,7 +842,11 @@
       <c r="H9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
@@ -820,7 +856,11 @@
       <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
@@ -830,7 +870,11 @@
       <c r="H11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
@@ -840,7 +884,11 @@
       <c r="H12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
@@ -850,7 +898,11 @@
       <c r="H13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
@@ -860,58 +912,58 @@
       <c r="H14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="8">
         <f>SUM(G3:G18)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP/攻击为初值 🔧。</t>
         </is>
@@ -1049,210 +1101,210 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="8">
         <f>SUM(I3:I18)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>总攻击 = 基础攻击 + 武器加成,投掷对应面数骰(如总攻击8→d8)。角色协同/特殊效果按牌自由填写。强武器建议只放中心。</t>
         </is>
@@ -1373,150 +1425,150 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="8">
         <f>SUM(H3:H14)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>集齐若干碎片可拼成炸弹(附加行动埋下,下一轮爆炸),炸整区所有人。几片成弹/伤害 🔧 待定。</t>
         </is>
@@ -1654,186 +1706,186 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="8">
         <f>SUM(I3:I16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>食物:补充 HP。护甲:被攻击时消耗以反应式减伤(不给额外行动/抽牌)。中心物资最丰富。特殊效果列写附加功能。</t>
         </is>
@@ -1951,246 +2003,246 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>E01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>变异狼群</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr"/>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>目标区所有人受 2 点攻击</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="G3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>E02</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>洪水</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr"/>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>目标区所有人弃掉手上的武器牌(已装备的除外)</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G4" s="9" t="n">
+      <c r="G4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>猴群</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>抢走目标区已装备的武器</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>已知事件</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="8">
         <f>SUM(G3:G17)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>随机事件在特定轮触发(🔧 4/6/7/9 待商榷)。触发时先掷 d4 定受影响外区,再抽事件牌。描述列写风味文字。</t>
         </is>
@@ -2286,272 +2338,388 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Myrtle</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr"/>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>You are not afraid of death. You are here to make a statement. If you are the first one to die, you win.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>最先牺牲(第一个被淘汰)即胜</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Social Butterfly</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr"/>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>游戏结束时正确认出特殊角色(Lover/Vendetta/Bodyguard)即胜</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="n">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>You are a social butterfly and is good at observing the relationships among people. If at the end of the game, you correctly identified 3 other secret identities, you win.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>游戏结束时正确认出3个特殊角色(Lover/Vendetta/Bodyguard)即胜</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>需推理身份</t>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>需推理身份。❓ 限定这三种角色,还是任意 3 名其他玩家的身份?(限定时可能不在场)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Lover(爱人)</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>爱上左边的玩家;若左边玩家获胜,爱人也胜</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="n">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Star-crossed Lovers</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>You fell in love with the second tribute left of you. If that person wins, you win.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>爱上左边第二位玩家;若该玩家获胜,爱人也胜,两人可以同时获胜。</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>✅ 共 2 张 Lovers 卡,各自爱上自己左边第二位玩家。爱上的玩家也可以靠抽号决定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Sour Lemon</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>You hold a sour hatred for all lovers. If you can identify the lovers and kill one of them, you win.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>认出并杀死一名持有 Lovers 卡的玩家即胜</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>左右靠抽号决定</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>H04</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Sour Lemon</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>认出并杀死一名 Lover 即胜</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="n">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>与 Lovers 联动。目标 = 持 Lovers 卡者(不含被爱的人)。❓ 成对发牌:Lovers 不在场时如何处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Warrior</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>You are a warrior born to fight in the Arena. You want to show your strength and bring glory to your hometown. If you are the one that kills most tributes, you win.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>杀敌数最多即胜</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>与 Lover 联动</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>H05</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Warrior</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr"/>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>杀敌数最多即胜</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="n">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>对家:Pacifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>H06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Bodyguard</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>You are hired as the protector of the target of Vendetta. If the target survives or if you kill the Vendetta tribute, you win.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>保护 Vendetta 的复仇对象,使其不被杀(必须在结束时指出复仇对象);或杀死 Vendetta 的角色。</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>H06</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Bodyguard</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>保护 Vendetta 的复仇对象,使其不被杀</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="n">
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>与 Vendetta 联动。❓ 成对发牌:Vendetta 不在场时如何处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>H07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Vendetta</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>The father of the tribute on your right killed your family in a fight. You are here for vengeance. If you are the person that finishes this tribute, you win.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>杀死右边的玩家即胜。</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>与 Vendetta 联动</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>H07</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Vendetta</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>杀死右边的玩家才胜(唯一条件)</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="n">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>✅ 保留风险:目标被别人杀掉则无法获胜,无后备条件。需要杀死的玩家也可以靠抽号决定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>H08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Pacifier</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>You have a mission of peace. If you are the last 3 people that survives without using violence, you win.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>进入最后三名存活玩家的那一刻,若整局从未主动攻击,即胜;达成后可自由使用武力。</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>左右靠抽号决定</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>✅ 中心强制攻击不算主动攻击;埋炸弹算使用武力。对家:Warrior</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>H09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Collector</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>You are a fervent weapon collector. If you die with 3 advance weapons, you win.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>如果死时有三件高级武器即获胜。</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>❓ 待定义『高级武器』(例:攻击 +3 及以上)。洪水事件是它的克星。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Negotiator</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>You are an expert negotiator. If you successfully exchange cards with everybody, you win.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>与至少(玩家人数 − 2)名不同玩家各完成一次双向交换手牌,即获胜。(单向给牌不算)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>🔧 N = 玩家人数 − 2,可改为 − 1。对家:Judas</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Judas(叛徒)</t>
+        </is>
+      </c>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>(提案)与同一名玩家在两个不同回合都完成过双向交换,之后亲手淘汰该玩家,且你自己存活到游戏结束。</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>❓ 提案版本,难度待定,见讨论。对家:Negotiator</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>数量合计</t>
         </is>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="8">
         <f>SUM(E3:E19)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>每位玩家秘密持有 1 张。允许多位胜者:各自对照身份结算。描述列写风味文字;完整清单/数量 ❓ 待补。</t>
         </is>

</xml_diff>

<commit_message>
docs: mutual Lovers pair, Social Butterfly any-3, Judas = kill a 3x trade partner
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>游戏结束时正确认出3个特殊角色(Lover/Vendetta/Bodyguard)即胜</t>
+          <t>游戏结束时正确认出任意 3 名其他玩家的隐藏身份即胜(Lovers 这一对算 1 个)。</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>需推理身份。❓ 限定这三种角色,还是任意 3 名其他玩家的身份?(限定时可能不在场)</t>
+          <t>✅ 任意 3 个隐藏身份;认出 Lovers 这一对只算 1 个。</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>You fell in love with the second tribute left of you. If that person wins, you win.</t>
+          <t>You and another tribute are star-crossed lovers. If your lover wins, you win.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>爱上左边第二位玩家;若该玩家获胜,爱人也胜,两人可以同时获胜。</t>
+          <t>两张相同的 Lovers 牌,持有者互相爱上;任一方获胜,另一方也胜,两人可以同时获胜。</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>✅ 共 2 张 Lovers 卡,各自爱上自己左边第二位玩家。爱上的玩家也可以靠抽号决定。</t>
+          <t>✅ 2 张相同的牌,成对发出。风味文字按新规则改过,可再润色。❓ 开局两人是否知道对方是谁?</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>认出并杀死一名持有 Lovers 卡的玩家即胜</t>
+          <t>认出并杀死两名 Lovers 中的任意一人即胜</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>与 Lovers 联动。目标 = 持 Lovers 卡者(不含被爱的人)。❓ 成对发牌:Lovers 不在场时如何处理</t>
+          <t>与 Lovers 联动。❓ Lovers 不在场时如何处理</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>(提案)与同一名玩家在两个不同回合都完成过双向交换,之后亲手淘汰该玩家,且你自己存活到游戏结束。</t>
+          <t>亲手淘汰一名和你双向交换过 3 次手牌的玩家,即胜。</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>❓ 提案版本,难度待定,见讨论。对家:Negotiator</t>
+          <t>✅ 3 次交换须是同一个人。不需要活到最后。对家:Negotiator</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: strict ties for Myrtle/Warrior; Pacifier moves to 11+, Social Butterfly joins the 5-player base
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -2361,7 +2361,11 @@
       <c r="E3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>✅ 首批死亡有多人(同回合结算)时不算胜</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2471,7 +2475,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>杀敌数最多即胜</t>
+          <t>杀敌数唯一最多即胜</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -2479,7 +2483,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>对家:Pacifier</t>
+          <t>✅ 并列最多不算胜。对家:Pacifier</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2573,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>✅ 中心强制攻击不算主动攻击;埋炸弹算使用武力。对家:Warrior</t>
+          <t>✅ 中心强制攻击不算主动攻击;埋炸弹算使用武力。✅ 推荐 11 人以上才加入。对家:Warrior</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: rename Pacifier -> Pacifist
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -2483,7 +2483,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>✅ 并列最多不算胜。对家:Pacifier</t>
+          <t>✅ 并列最多不算胜。对家:Pacifist</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pacifier</t>
+          <t>Pacifist</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: add 推荐身份配置 sheet to deck workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物资(食物·护甲)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="随机事件" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="隐藏身份" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="推荐身份配置" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2737,4 +2738,184 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>身份配置</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>这一档变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Warrior、Vendetta、Bodyguard、Myrtle、Social Butterfly</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张 + Negotiator</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>加 Negotiator</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张 + Lovers×2</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Negotiator 换成 Lovers 一对(成对加入)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>7 人配置 + Sour Lemon</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Lovers 的克星</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>8 人配置 + Pacifist</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>进前三才难,苟着不再稳赢</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>9 人配置 + Negotiator</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Negotiator 回归</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>10 人配置 + Collector</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>全部 12 张 + Judas</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>长局回合多,最易达成 3 次交换</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>发牌规则:每人 1 张身份,N 人局从 12 张中选 N 张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Lovers 两张必须一起放;Sour Lemon 只在 Lovers 在场时放;Bodyguard 只和 Vendetta 一起放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 玩家可自由调整,以上仅为推荐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>平局从严:Myrtle 首批死亡多人、Warrior 杀敌数并列,均不算胜。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sync 8 random events from Numbers, add The Feast flavor text
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1908,7 +1908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2014,7 +2014,11 @@
           <t>变异狼群</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Roaring, muted wolves are released into the zone. You fight them with all you have. *Health -4</t>
+        </is>
+      </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
@@ -2022,7 +2026,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>目标区所有人受 2 点攻击</t>
+          <t>目标区所有人受 4点攻击</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -2031,7 +2035,7 @@
         </is>
       </c>
       <c r="G3" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
@@ -2050,7 +2054,11 @@
           <t>洪水</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Water seeped in from the ground and rose until it washed everything away… *Loses every card except for the equipped weapons.</t>
+        </is>
+      </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
@@ -2067,7 +2075,7 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
@@ -2086,7 +2094,11 @@
           <t>猴群</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>A gigantic ape appears and took your weapon. Startled, you watch as it disappears into the woods. *Lose equipped weapon</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
           <t>掷d4</t>
@@ -2103,7 +2115,7 @@
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
@@ -2112,54 +2124,164 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>沙尘暴</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>遮天蔽日的黄沙遮挡了所有人的视线。本轮无法移动区域。</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>掷d4</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>目标区角色本轮无法移动区域。</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>和平日</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Everyone await with bated breath but nothing happens —- the game maker seems to be in a good mood. Lucky you!</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>掷d4</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Fire Balls</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Bolts of fire balls shoot at you from the sky. You scream, run and hide, but still get burned. *Health -3</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Every zone except for zone 1 and the water zone.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>目标区所有人受 3点攻击</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Hungry Dogs</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>A pack of hungry dogs raided the area. If you have food for exchange, you are left alone. *Loses 2 food cards OR Health -3.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>掷d4</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Loses 2 food cards OR Health -3.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>The Feast</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>The game maker spreads a feast at the heart of the Arena — weapons, food, riches for the taking. Hunger pulls you in, and so does everyone else. *Draw 2 extra cards if you are in the central zone this round.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>本回合在中心区的人多抽 2 张牌</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -2231,29 +2353,39 @@
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
     </row>
-    <row r="19">
-      <c r="F19" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="G19" s="8">
-        <f>SUM(G3:G17)</f>
+      <c r="G20" s="8">
+        <f>SUM(G3:G18)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>随机事件在特定轮触发(🔧 4/6/7/9 待商榷)。触发时先掷 d4 定受影响外区,再抽事件牌。描述列写风味文字。</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23"/>
+    <row r="24"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A21:F23"/>
+    <mergeCell ref="A22:F24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: The Feast resolves next round (events fire after movement); record event timing rule
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>The game maker spreads a feast at the heart of the Arena — weapons, food, riches for the taking. Hunger pulls you in, and so does everyone else. *Draw 2 extra cards if you are in the central zone this round.</t>
+          <t>The game maker spreads a feast at the heart of the Arena — weapons, food, riches for the taking. Hunger pulls you in, and so does everyone else. *Next round, draw 2 extra cards if you end in the central zone.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -2274,14 +2274,18 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>本回合在中心区的人多抽 2 张牌</t>
+          <t>下回合在中心区的人多抽 2 张牌(本回合预告)</t>
         </is>
       </c>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="5" t="n"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>唯一预告型事件:本回合公布,下回合生效,给玩家一轮谈判与布局。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>

</xml_diff>

<commit_message>
feat: 12 characters + trident/bow in deck table; loader reads HP header and zone names
- characters C01-C12 (user's 8 + Bram/Iris/Mira/Wren), Natalie poison-card mechanic,
  Riley steals hand cards only; HP scale 11/13/15
- loader: 'HP' column (legacy 'HP档(3/5/7)' still accepted); 林区/水区/石区/城区/Central
- rules: outer ring order 林 -> 水 -> 石 -> 城

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>HP档(3/5/7)</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>3</v>
@@ -746,15 +746,27 @@
           <t>C01</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Riley</t>
+        </is>
+      </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Growing up in a poor neighbourhood, you found ways to fit into the shadow and feed yourself without other’s noticeable.</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+          <t>Growing up in a poor neighbourhood, Riley found ways to fit into the shadow and feed yourself without other’s notice.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>小偷：每回合可以选择一个附加动作——偷取同区域一名玩家的卡牌。投掷4面骰子，如果是4则成功，随机抽取一张对方卡牌；1-3则失败。（只能偷手牌，不能偷已装备的武器）</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
@@ -764,11 +776,27 @@
           <t>C02</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Elliot</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Growing up in the local market, Elliot started to search and collect things to sell since he was a kid —- deserted shoes, books, teddy bears… “The unseen treasures around us”, he calls them. </t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>如果同区域无人，一次可以捡两张卡，并且最多可以有6张手牌。</t>
+        </is>
+      </c>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
@@ -778,11 +806,27 @@
           <t>C03</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Agatha</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Agatha worked in a manufacturing factory as a girl, and learned to make weapons out of simple objects.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>可以将两张初级武器组合使用，做成攻击力更高的武器或护盾。</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
@@ -792,11 +836,27 @@
           <t>C04</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Fae</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fae is small but very agile. She is not a master of the fight, but a master of hide and seek.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>在林区攻击的回合也可以拿一张手牌。</t>
+        </is>
+      </c>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
     </row>
@@ -806,13 +866,33 @@
           <t>C05</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Natalie</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Although being raised in the city, Natalie preferred being in nature. She believes there is more power in nature than people can see.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>下毒：可以用 2 张食物牌换 1 张毒食物牌（背面与普通食物相同，由 Natalie 私下保管），并洗入所在区域的牌堆。抽到毒食物的人 Health -4。</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>✅ 采用毒食物牌方案，需要制作若干张毒食物牌</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -820,11 +900,27 @@
           <t>C06</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Cato</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Cato was training to be in the Arena since he was a kid. It is his dream to bring glory to his hometown by winning the game.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>因为Cato所在的城市离首都太近，他们被禁止学习科技，因此Cato无法使用碎片拼成炸药。</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
     </row>
@@ -834,11 +930,27 @@
           <t>C07</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Garcia</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Garcia is not the strongest of the tributes, but she is the smartest.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>只需要2枚碎片就可以制成一个炸药。</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
     </row>
@@ -848,11 +960,27 @@
           <t>C08</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Tobias</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Growing up near the water, Tobias learned from a very young age how to use the trident, both as a formidable weapon and to fish.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>如果拿到三叉戟，在水区每回合可以多拿一张手牌。</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
     </row>
@@ -862,13 +990,33 @@
           <t>C09</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Bram</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Bram spent his youth hauling stone in the quarries. He is slow, but the mountain taught him to endure what others cannot.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>在石区时，每次受到攻击的伤害 -1。</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>石区专属，防守型</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -876,13 +1024,33 @@
           <t>C10</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Iris</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Iris ran messages through the city's back alleys for anyone who paid. She knows secrets — and knows what they are worth.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>在城区时，每局一次，可以秘密查看同区域一名玩家的隐藏身份。</t>
+        </is>
+      </c>
       <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>城区专属，信息型；信息很强，限每局一次</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -890,13 +1058,33 @@
           <t>C11</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Mira learned herbs from her grandmother. In the Arena, she knows a meal can buy more than strength — it can buy loyalty.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>附加行动：可以把自己的食物给同区域另一名玩家吃，回血效果 +2。</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>帮盟友型；bot 不会用，需要 agent</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -904,13 +1092,33 @@
           <t>C12</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Wren</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Wren hunted with her father in the northern woods. She never misses — as long as she has a bow.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>拿到弓时，可以攻击相邻区域的玩家。</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>远程型；需要武器表里的『弓』</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -966,7 +1174,7 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP/攻击为初值 🔧。</t>
+          <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP 量级 11/13/15、攻击 2/3/4,均为初值 🔧。</t>
         </is>
       </c>
     </row>
@@ -986,7 +1194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1102,28 +1310,92 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>W01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>三叉戟</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>A long, three-pronged spear — as good for fishing as it is for fighting.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>装备</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>水区</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Tobias：在水区每回合多拿一张手牌</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>🔧 攻击加成、张数待定</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>W02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>弓</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>A hunter's bow, light and silent. In the right hands, distance is a weapon.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>装备</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>林区</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Wren：可攻击相邻区域的玩家</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>🔧 攻击加成、张数待定</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -1293,29 +1565,53 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="6" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+    </row>
     <row r="20">
-      <c r="H20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="I20" s="8">
-        <f>SUM(I3:I18)</f>
+      <c r="I22" s="8">
+        <f>SUM(I3:I20)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>总攻击 = 基础攻击 + 武器加成,投掷对应面数骰(如总攻击8→d8)。角色协同/特殊效果按牌自由填写。强武器建议只放中心。</t>
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:F24"/>
+    <mergeCell ref="A24:F26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: deck table organized per zone (one sheet per zone)
Replace the 武器/弹药碎片/物资 sheets with 林区/水区/石区/城区/中心牌堆. Each row
is one card design with 类型/数值/张数 for that zone. Loader reads the zone
sheets, rejects unknown card types with a clear message, and reads armor
written as -2 as a reduction of 2. Tests share an xlsx fixture helper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人物" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武器" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="弹药碎片" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物资(食物·护甲)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="随机事件" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="隐藏身份" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="推荐身份配置" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="林区牌堆" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水区牌堆" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="石区牌堆" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城区牌堆" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中心牌堆" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="随机事件" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="隐藏身份" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="推荐身份配置" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -572,28 +574,28 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>三个常问的列写在哪:</t>
+          <t>牌堆按区分:林区牌堆 / 水区牌堆 / 石区牌堆 / 城区牌堆 / 中心牌堆,每区一张表。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 描述       = 每张牌的风味文字(例:名字『蘑菇』,描述『看上去有点毒的蘑菇』)。</t>
+          <t xml:space="preserve">  • 一行 = 一种牌;张数 = 这种牌在本区牌堆里放几张。通用牌(如面包)在几个区都有,就在几张表里各写一行。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 角色协同   = 某牌在特定角色手里更强(例:『刺客手中额外+2 攻击』)。</t>
+          <t xml:space="preserve">  • 类型只能填:武器 / 食物 / 护甲 / 碎片。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 特殊效果   = 附加功能(例:『击杀时抽 1 张食物』『使用后可再移动一次』)。</t>
+          <t xml:space="preserve">  • 数值:武器 = 攻击加成;食物 = 回血;护甲 = 减伤(写 2 或 -2 都行);碎片 = 1。</t>
         </is>
       </c>
     </row>
@@ -603,28 +605,28 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>牌数起始建议(6 人局,约 55 张物资;可按玩家数×8~10 缩放):</t>
+          <t>三个常问的列写在哪:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 外区每区 ≈ 9 张:武器2(弱)/食物4/护甲3</t>
+          <t xml:space="preserve">  • 描述       = 每张牌的风味文字(例:名字『蘑菇』,描述『看上去有点毒的蘑菇』)。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 中心 ≈ 11 张:武器6(含强武器+3/+4)/食物3/护甲2</t>
+          <t xml:space="preserve">  • 角色协同   = 某牌在特定角色手里更强(例:『刺客手中额外+2 攻击』)。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 强武器只放中心;食物/护甲别过多,否则战斗打不死人、拖慢节奏。</t>
+          <t xml:space="preserve">  • 特殊效果   = 附加功能(例:『击杀时抽 1 张食物』『使用后可再移动一次』)。</t>
         </is>
       </c>
     </row>
@@ -634,7 +636,218 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>牌数起始建议(6 人局,约 55 张物资;可按玩家数×8~10 缩放):</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 外区每区 ≈ 9 张:武器2(弱)/食物4/护甲3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 中心 ≈ 11 张:武器6(含强武器+3/+4)/食物3/护甲2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 强武器只放中心;食物/护甲别过多,否则战斗打不死人、拖慢节奏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>标注约定:✅ 已确认  🔧 初值待测  ❓ 待定。数值以模拟/试玩结果为准。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>身份配置</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>这一档变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Warrior、Vendetta、Bodyguard、Myrtle、Social Butterfly</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张 + Negotiator</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>加 Negotiator</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>基础 5 张 + Lovers×2</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Negotiator 换成 Lovers 一对(成对加入)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>7 人配置 + Sour Lemon</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Lovers 的克星</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>8 人配置 + Pacifist</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>进前三才难,苟着不再稳赢</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>9 人配置 + Negotiator</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Negotiator 回归</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>10 人配置 + Collector</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>全部 12 张 + Judas</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>长局回合多,最易达成 3 次交换</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>发牌规则:每人 1 张身份,N 人局从 12 张中选 N 张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Lovers 两张必须一起放;Sour Lemon 只在 Lovers 在场时放;Bodyguard 只和 Vendetta 一起放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 玩家可自由调整,以上仅为推荐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>平局从严:Myrtle 首批死亡多人、Warrior 杀敌数并列,均不算胜。</t>
         </is>
       </c>
     </row>
@@ -1194,19 +1407,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1217,45 +1429,40 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>武器名</t>
+          <t>类型</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>牌名</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>攻击加成(+X)</t>
-        </is>
-      </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>类型(装备/一次性)</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>所在区域牌堆</t>
+          <t>角色协同</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>角色协同</t>
+          <t>特殊效果</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>特殊效果</t>
+          <t>张数</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>张数</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1264,138 +1471,87 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>示例↓ W01</t>
+          <t>示例↓ 林00</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>示例·猎刀</t>
+          <t>食物</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>一把磨得发亮的短刀</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
+          <t>蘑菇</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>看上去有点毒的蘑菇</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>装备</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>任意/外区</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>刺客手中额外+2</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>击杀时抽1张食物</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="n">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>攻击叠加到基础攻击上</t>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>格式示例</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>W01</t>
+          <t>林01</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>三叉戟</t>
+          <t>武器</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>A long, three-pronged spear — as good for fishing as it is for fighting.</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>装备</t>
-        </is>
+          <t>弓</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>A hunter's bow, light and silent. In the right hands, distance is a weapon.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>水区</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Tobias：在水区每回合多拿一张手牌</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n">
+          <t>Wren:拿到弓时可攻击相邻区域的玩家</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>🔧 攻击加成、张数待定</t>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>🔧 数值、张数待定</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>W02</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>弓</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>A hunter's bow, light and silent. In the right hands, distance is a weapon.</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>装备</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>林区</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Wren：可攻击相邻区域的玩家</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>🔧 攻击加成、张数待定</t>
-        </is>
-      </c>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -1407,7 +1563,6 @@
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -1419,7 +1574,6 @@
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
       <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -1431,7 +1585,6 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -1443,7 +1596,6 @@
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
       <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -1455,7 +1607,6 @@
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
       <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -1467,7 +1618,6 @@
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -1479,7 +1629,6 @@
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -1491,7 +1640,6 @@
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -1503,7 +1651,6 @@
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -1515,7 +1662,6 @@
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -1527,7 +1673,6 @@
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -1539,7 +1684,6 @@
       <c r="G16" s="6" t="n"/>
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -1551,67 +1695,30 @@
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
       <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="H22" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="I22" s="8">
-        <f>SUM(I3:I20)</f>
+      <c r="H19" s="8">
+        <f>SUM(H3:H17)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>总攻击 = 基础攻击 + 武器加成,投掷对应面数骰(如总攻击8→d8)。角色协同/特殊效果按牌自由填写。强武器建议只放中心。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26"/>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A24:F26"/>
+    <mergeCell ref="A21:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1623,17 +1730,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1645,27 +1752,27 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>碎片名</t>
+          <t>类型</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>牌名</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>集齐需求(几片)</t>
-        </is>
-      </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>炸弹伤害</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>影响范围</t>
+          <t>角色协同</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -1687,50 +1794,76 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>示例↓ F01</t>
+          <t>示例↓ 水00</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>示例·弹药碎片</t>
+          <t>食物</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>锈迹斑斑的金属零件</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
+          <t>鱼</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>刚从水里捞上来的鱼</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>整个区域所有人</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>附加行动埋下,下一轮爆炸</t>
+          <t>格式示例</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>水01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>三叉戟</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>A long, three-pronged spear — as good for fishing as it is for fighting.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Tobias:在水区每回合多拿一张手牌</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>🔧 数值、张数待定</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -1853,29 +1986,62 @@
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+    </row>
     <row r="16">
-      <c r="G16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H16" s="8">
-        <f>SUM(H3:H14)</f>
+      <c r="H19" s="8">
+        <f>SUM(H3:H17)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>集齐若干碎片可拼成炸弹(附加行动埋下,下一轮爆炸),炸整区所有人。几片成弹/伤害 🔧 待定。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A18:F20"/>
+    <mergeCell ref="A21:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1887,19 +2053,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1910,45 +2075,40 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>牌名</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>描述</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>类型(食物/护甲)</t>
-        </is>
-      </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>效果</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>角色协同</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>所在区域牌堆</t>
+          <t>特殊效果</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>特殊效果</t>
+          <t>张数</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>张数</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1957,48 +2117,35 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>示例↓ S01</t>
+          <t>示例↓ 石00</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>蘑菇</t>
+          <t>护甲</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>看上去有点毒的蘑菇</t>
+          <t>石板盾</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>食物</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>回复 HP</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="n">
+          <t>一块沉重的石板</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>任意</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>被某角色食用无副作用</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>回血数值待定</t>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>格式示例</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2159,6 @@
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
       <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -2024,7 +2170,6 @@
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
       <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -2036,7 +2181,6 @@
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -2048,7 +2192,6 @@
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
       <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -2060,7 +2203,6 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -2072,7 +2214,6 @@
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
       <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -2084,7 +2225,6 @@
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
       <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -2096,7 +2236,6 @@
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -2108,7 +2247,6 @@
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -2120,7 +2258,6 @@
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -2132,7 +2269,6 @@
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -2144,7 +2280,6 @@
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -2156,7 +2291,6 @@
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -2168,23 +2302,22 @@
       <c r="G16" s="6" t="n"/>
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="H18" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="I18" s="8">
-        <f>SUM(I3:I16)</f>
+      <c r="H18" s="8">
+        <f>SUM(H3:H16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>食物:补充 HP。护甲:被攻击时消耗以反应式减伤(不给额外行动/抽牌)。中心物资最丰富。特殊效果列写附加功能。</t>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
         </is>
       </c>
     </row>
@@ -2199,6 +2332,574 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>牌名</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>角色协同</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>特殊效果</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>张数</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>示例↓ 城00</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>铁管</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>从废墟里拆下来的铁管</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>格式示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>张数合计</t>
+        </is>
+      </c>
+      <c r="H18" s="8">
+        <f>SUM(H3:H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A20:F22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>牌名</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>角色协同</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>特殊效果</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>张数</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>示例↓ 中00</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>步枪</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>保养良好的军用步枪</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>格式示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>张数合计</t>
+        </is>
+      </c>
+      <c r="H18" s="8">
+        <f>SUM(H3:H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。中心物资最丰富,建议约 11 张:武器 6(含 +3/+4 强武器)、食物 3、护甲 2。强武器只放中心;中心强制开战。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A20:F22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2691,7 +3392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3170,184 +3871,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>人数</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>身份配置</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>这一档变化</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Warrior、Vendetta、Bodyguard、Myrtle、Social Butterfly</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>基础 5 张</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>基础 5 张 + Negotiator</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>加 Negotiator</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>基础 5 张 + Lovers×2</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Negotiator 换成 Lovers 一对(成对加入)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>7 人配置 + Sour Lemon</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Lovers 的克星</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>8 人配置 + Pacifist</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>进前三才难,苟着不再稳赢</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>9 人配置 + Negotiator</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Negotiator 回归</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>10 人配置 + Collector</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>全部 12 张 + Judas</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>长局回合多,最易达成 3 次交换</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>发牌规则:每人 1 张身份,N 人局从 12 张中选 N 张。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Lovers 两张必须一起放;Sour Lemon 只在 Lovers 在场时放;Bodyguard 只和 Vendetta 一起放。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • 玩家可自由调整,以上仅为推荐。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>平局从严:Myrtle 首批死亡多人、Warrior 杀敌数并列,均不算胜。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: special (character-synergy) weapons live in the center deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1407,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1504,43 +1504,15 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>林01</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>武器</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>弓</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>A hunter's bow, light and silent. In the right hands, distance is a weapon.</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Wren:拿到弓时可攻击相邻区域的玩家</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>🔧 数值、张数待定</t>
-        </is>
-      </c>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -1685,40 +1657,29 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="G19" s="7" t="inlineStr">
+    <row r="18">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H19" s="8">
-        <f>SUM(H3:H17)</f>
+      <c r="H18" s="8">
+        <f>SUM(H3:H16)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
-        </is>
-      </c>
-    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22"/>
-    <row r="23"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A21:F23"/>
+    <mergeCell ref="A20:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1730,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1827,43 +1788,15 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>水01</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>武器</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>三叉戟</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>A long, three-pronged spear — as good for fishing as it is for fighting.</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Tobias:在水区每回合多拿一张手牌</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>🔧 数值、张数待定</t>
-        </is>
-      </c>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -2008,40 +1941,29 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="G19" s="7" t="inlineStr">
+    <row r="18">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H19" s="8">
-        <f>SUM(H3:H17)</f>
+      <c r="H18" s="8">
+        <f>SUM(H3:H16)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
-        </is>
-      </c>
-    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22"/>
-    <row r="23"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A21:F23"/>
+    <mergeCell ref="A20:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2317,7 +2239,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2523,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。</t>
+          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2718,26 +2640,82 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>中01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>弓</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>A hunter's bow, light and silent. In the right hands, distance is a weapon.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Wren:拿到弓时可攻击相邻区域的玩家</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>特殊武器。🔧 数值、张数待定</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>中02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>三叉戟</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>A long, three-pronged spear — as good for fishing as it is for fighting.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Tobias:在水区每回合多拿一张手牌</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>特殊武器。🔧 数值、张数待定</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -2871,29 +2849,51 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
     <row r="18">
-      <c r="G18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H16)</f>
+      <c r="H20" s="8">
+        <f>SUM(H3:H18)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。中心物资最丰富,建议约 11 张:武器 6(含 +3/+4 强武器)、食物 3、护甲 2。强武器只放中心;中心强制开战。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>类型只能填 武器/食物/护甲/碎片。中心物资最丰富,建议约 11 张:武器 6(含 +3/+4 强武器)、食物 3、护甲 2。强武器和所有特殊武器(有角色协同的)只放中心;中心强制开战。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A22:F24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: fill five zone decks (12 cards per outer zone), weapon tiers, bomb = 4 fragments
- import user's cards from Numbers; fill 类型/数值/张数; add armor & a few themed cards
- 类型 column gets a dropdown (武器/食物/护甲/碎片)
- loader reads values written as text (+2Health, +2 防御)
- rules: outer = basic weapons, center = advanced; city has fragments, stone has armor

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1407,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1504,81 +1504,225 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>林01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>蘑菇</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>不知道有没有毒的蘑菇</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>林02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>红果子</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>闻上去香香的</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>林03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>死兔子</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>看上去死去不久的兔子</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>林04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>苹果</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>一个完美的苹果！</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>林05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>木棍</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>一根粗壮的木棍</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>林06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>树杈</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>一根可怜的小树杈</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>林07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>树皮甲</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>用树皮和藤蔓绑成的护甲，聊胜于无</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -1657,30 +1801,112 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
     <row r="18">
-      <c r="G18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H16)</f>
+      <c r="H25" s="8">
+        <f>SUM(H3:H23)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A27:F29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+      <formula1>"武器,食物,护甲,碎片"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1691,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1788,81 +2014,225 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>水01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>鱼</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>刚从水里捞上来的鱼</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>水02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>虾</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>一只蹦哒的小虾</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>水03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>章鱼</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>这只章鱼被太阳晒得软趴趴的</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>水04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>贝壳</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>砸一下就能吃到肉，可惜不多</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>水05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>绳子</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>海藻缠绕形成的绳子，可以甩着玩</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>水06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>木桨</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>一根完整的船桨</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>水07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>龟壳</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>一块被遗弃的龟壳，刚好能挡在胸前</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -1941,30 +2311,112 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
     <row r="18">
-      <c r="G18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H16)</f>
+      <c r="H25" s="8">
+        <f>SUM(H3:H23)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A27:F29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+      <formula1>"武器,食物,护甲,碎片"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1975,7 +2427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2072,81 +2524,241 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>石01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>石板盾</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>一块沉重的石板</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>石02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>岩石护臂</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>用碎石和皮绳做成的护臂</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>石03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>矿工头盔</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>一顶凹了一块的旧头盔，灯早就不亮了</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>石04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>石头</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>只是一块石头</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>石05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>燧石片</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>一片锋利的燧石，小心别割到自己</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>石06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>苔藓</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>长在石缝里的苔藓，勉强能吃</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>石07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>肉干</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>不知道谁留下的肉干，硬得像石头</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -2225,30 +2837,112 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
     <row r="18">
-      <c r="G18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H16)</f>
+      <c r="H25" s="8">
+        <f>SUM(H3:H23)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A27:F29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+      <formula1>"武器,食物,护甲,碎片"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2259,7 +2953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2356,81 +3050,229 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>城01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>方便面</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>一般般好吃的方便面</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>城02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>西红柿</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>软掉的西红柿，好像快烂了</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>城03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>死老鼠</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>这也可以吃吗？</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>城04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>汉堡</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>被小动物咬了一口的汉堡</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>城05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>铁管</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>从废墟里拆下来的铁管</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>城06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>车牌</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>一块掉落的车牌</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>城07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>碎片</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>电器碎片</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>看上去有些电路还没损坏——或许可以用来做点什么？</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>需要4张合成一个炸弹</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>碎片只在城区出现</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -2509,30 +3351,112 @@
       <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
     <row r="18">
-      <c r="G18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H16)</f>
+      <c r="H25" s="8">
+        <f>SUM(H3:H23)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。张数 = 这张牌在本区牌堆里放几张。外区建议约 9 张:武器 2(弱)、食物 4、护甲 3,可加少量碎片。特殊武器(有角色协同的)不放外区,统一放中心。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F22"/>
+    <mergeCell ref="A27:F29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+      <formula1>"武器,食物,护甲,碎片"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2543,7 +3467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2661,7 +3585,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -2674,7 +3598,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>特殊武器。🔧 数值、张数待定</t>
+          <t>特殊武器</t>
         </is>
       </c>
     </row>
@@ -2700,7 +3624,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -2713,119 +3637,347 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>特殊武器。🔧 数值、张数待定</t>
+          <t>特殊武器</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>中03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>长剑</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>一把寒光闪闪的长剑，拿在手里沉甸甸的</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>描述由 Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>中04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>斧子</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>一把磨得锋利的伐木斧</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>描述由 Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>中05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>弯刀</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>刀刃弯如新月，据说曾属于一位不肯倒下的战士</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>在角色死亡时会对对手造成3点伤害</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>对手 = 击杀持有者的人。描述由 Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>中06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>双节棍</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>甩起来呼呼作响——希望别打到自己</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>描述由 Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>中07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>西瓜</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>解渴且香甜的新鲜西瓜，让人一扫疲惫</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>中08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>鸡腿</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>鲜嫩多汁的烤鸡腿</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>中09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>南瓜派</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>香喷喷热腾腾的南瓜派</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>中10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>食物</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>牛排</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>滴着黄油的烤牛排</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>中11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>防弹背心</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>军用防弹背心，有点大但很结实</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>中12</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>钢盔</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>一顶锃亮的钢盔</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -2871,30 +4023,145 @@
       <c r="H18" s="6" t="n"/>
       <c r="I18" s="6" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+    </row>
     <row r="20">
-      <c r="G20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H20" s="8">
-        <f>SUM(H3:H18)</f>
+      <c r="H30" s="8">
+        <f>SUM(H3:H28)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>类型只能填 武器/食物/护甲/碎片。中心物资最丰富,建议约 11 张:武器 6(含 +3/+4 强武器)、食物 3、护甲 2。强武器和所有特殊武器(有角色协同的)只放中心;中心强制开战。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24"/>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>中心全是高级武器(+3/+4)和所有特殊武器;食物更好(+3/+4)。中心强制开战。类型用下拉菜单选:武器/食物/护甲/碎片。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:F24"/>
+    <mergeCell ref="A32:F34"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+      <formula1>"武器,食物,护甲,碎片"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3737,7 +5004,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>❓ 待定义『高级武器』(例:攻击 +3 及以上)。洪水事件是它的克星。</t>
+          <t>✅ 高级武器 = 中心牌堆里的武器(+3/+4)。洪水事件是它的克星。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: city deck +1 electronic fragment (6), -1 food (tomato)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -2953,7 +2953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3083,7 +3083,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>城02</t>
+          <t>城03</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>西红柿</t>
+          <t>死老鼠</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>软掉的西红柿，好像快烂了</t>
+          <t>这也可以吃吗？</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -3114,7 +3114,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>城03</t>
+          <t>城04</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -3124,16 +3124,16 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>死老鼠</t>
+          <t>汉堡</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>这也可以吃吗？</t>
+          <t>被小动物咬了一口的汉堡</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
@@ -3145,22 +3145,22 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>城04</t>
+          <t>城05</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>食物</t>
+          <t>武器</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>汉堡</t>
+          <t>铁管</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>被小动物咬了一口的汉堡</t>
+          <t>从废墟里拆下来的铁管</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -3169,14 +3169,14 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>城05</t>
+          <t>城06</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -3186,12 +3186,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>铁管</t>
+          <t>车牌</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>从废墟里拆下来的铁管</t>
+          <t>一块掉落的车牌</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -3200,79 +3200,59 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>城06</t>
+          <t>城07</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>武器</t>
+          <t>碎片</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>车牌</t>
+          <t>电器碎片</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>一块掉落的车牌</t>
+          <t>看上去有些电路还没损坏——或许可以用来做点什么？</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>需要4张合成一个炸弹</t>
+        </is>
+      </c>
       <c r="H8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="5" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>碎片只在城区出现</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>城07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>碎片</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>电器碎片</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>看上去有些电路还没损坏——或许可以用来做点什么？</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>需要4张合成一个炸弹</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>碎片只在城区出现</t>
-        </is>
-      </c>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -3417,43 +3397,32 @@
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="G25" s="7" t="inlineStr">
+    <row r="24">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H25" s="8">
-        <f>SUM(H3:H23)</f>
+      <c r="H24" s="8">
+        <f>SUM(H3:H22)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A27:F29"/>
+    <mergeCell ref="A26:F28"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B3:B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
+    <dataValidation sqref="B3:B22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="类型" error="只能选 武器 / 食物 / 护甲 / 碎片" type="list">
       <formula1>"武器,食物,护甲,碎片"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: rename character Wren -> Micheal
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1307,12 +1307,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Wren</t>
+          <t>Micheal</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Wren hunted with her father in the northern woods. She never misses — as long as she has a bow.</t>
+          <t>Micheal hunted with her father in the northern woods. She never misses — as long as she has a bow.</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Wren:拿到弓时可攻击相邻区域的玩家</t>
+          <t>Micheal:拿到弓时可攻击相邻区域的玩家</t>
         </is>
       </c>
       <c r="G3" s="5" t="n"/>

</xml_diff>

<commit_message>
docs: fix spelling Micheal -> Michael
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1307,12 +1307,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Micheal</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Micheal hunted with her father in the northern woods. She never misses — as long as she has a bow.</t>
+          <t>Michael hunted with her father in the northern woods. She never misses — as long as she has a bow.</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Micheal:拿到弓时可攻击相邻区域的玩家</t>
+          <t>Michael:拿到弓时可攻击相邻区域的玩家</t>
         </is>
       </c>
       <c r="G3" s="5" t="n"/>

</xml_diff>

<commit_message>
feat: Bram skill -> ignore armor (蛮力), HP 15->11
Replaces the stone-zone damage reduction that stacked into a fortress. Bram now
counters armor-stacking instead of being unkillable.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1210,24 +1210,24 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Bram spent his youth hauling stone in the quarries. He is slow, but the mountain taught him to endure what others cannot.</t>
+          <t>Bram spent his youth hauling stone in the quarries. His blows carry the weight of the mountain — no armor holds against him.</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>在石区时，每次受到攻击的伤害 -1。</t>
+          <t>蛮力：攻击时无视对方护甲(护甲不减伤，也不被消耗)。</t>
         </is>
       </c>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>石区专属，防守型</t>
+          <t>进攻/克制防御流</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tune: character HP tiers -> 8/10/12 (faster games); agents' private docs now list their skill; character panel shows total attack (base+weapon) and skill
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>3</v>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>2</v>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>2</v>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>2</v>
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>2</v>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>4</v>
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>3</v>
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>3</v>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>2</v>
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>2</v>
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>2</v>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>3</v>
@@ -1373,6 +1373,7 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1384,6 +1385,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: slim the deck from 60 to 42 cards, food from 23 to 10
- outer zones 12 -> 8 cards (forest/water food 7->3, stone armor 7->4 and
  food 2->1, city fragments 6->4 and food 3->1); center 12 -> 10 (food 4->2).
  Weapons unchanged (20), so fights come sooner and decks run out mid-game
- deck loader: 张数 0 leaves a card out (kept in the sheet as a record);
  blank still means 1
- play: the planter's prompt shows their pending bomb; tolerate say entries
  written as [to, text] lists

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -636,7 +636,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>牌数起始建议(6 人局,约 55 张物资;可按玩家数×8~10 缩放):</t>
+          <t>当前牌数(6 人局,共 42 张):外区每区 8 张,中心 10 张;食物共 10 张。张数填 0 = 暂时移出牌堆。</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,6 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1385,7 +1384,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -1532,7 +1530,7 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="5" t="n"/>
     </row>
@@ -1563,7 +1561,7 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="n"/>
     </row>
@@ -1594,7 +1592,7 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="5" t="n"/>
     </row>
@@ -1625,9 +1623,13 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1880,6 +1882,7 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -1891,10 +1894,11 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+          <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2046,7 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="5" t="n"/>
     </row>
@@ -2073,7 +2077,7 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="n"/>
     </row>
@@ -2135,9 +2139,13 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2390,6 +2398,7 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2401,10 +2410,11 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+          <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2562,7 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" s="5" t="n"/>
     </row>
@@ -2583,7 +2593,7 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
@@ -2618,7 +2628,7 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
@@ -2719,11 +2729,11 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 暂时移出牌堆(2026-09 精简)</t>
         </is>
       </c>
     </row>
@@ -2916,6 +2926,7 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2927,10 +2938,11 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+          <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
@@ -3078,9 +3090,13 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -3140,9 +3156,13 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3237,7 +3257,7 @@
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
@@ -3399,6 +3419,7 @@
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -3410,10 +3431,11 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>四个外区每区 12 张(数量一致)。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
+          <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
@@ -3814,9 +3836,13 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3845,9 +3871,13 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -4104,6 +4134,7 @@
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -4115,6 +4146,7 @@
         <v/>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rules: Lovers win only if both survive; an empty-center Feast heals 3 instead
- Lovers: both must be alive at the end (a lone survivor wins only as the survivor);
  the game still ends at once when only the two Lovers are left
- the Feast: bonus center draws, or +3 HP (capped at max) once the center deck is
  empty; public feast_heal event
- prompt table, rules doc and deck sheet updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1882,7 +1882,6 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -1894,7 +1893,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -2398,7 +2396,6 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2410,7 +2407,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -2926,7 +2922,6 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2938,7 +2933,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -3419,7 +3413,6 @@
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -3431,7 +3424,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
@@ -4134,7 +4126,6 @@
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -4146,7 +4137,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
@@ -4541,7 +4531,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下回合在中心区的人多抽 2 张牌(本回合预告)</t>
+          <t>下回合在中心区的人多抽 2 张牌(本回合预告);中心牌堆空了就改为回 3 血(不超过上限)</t>
         </is>
       </c>
       <c r="F10" s="5" t="n"/>
@@ -4634,6 +4624,7 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4645,6 +4636,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -4819,7 +4811,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>两张相同的 Lovers 牌,持有者互相爱上;任一方获胜,另一方也胜,两人可以同时获胜。</t>
+          <t>两张相同的 Lovers 牌,持有者互相爱上;两人都活到最后才同赢(一方死了,另一方只能以普通存活者身份赢);只剩两名恋人时游戏立即结束。</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
@@ -5115,6 +5107,7 @@
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -5126,6 +5119,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: remove armor; Bram gets a heavy blow; stone becomes the weapon zone
- deck sheet: every armor card set to 0 (kept as a record); stone refilled with
  basic weapons (石头 x3, 燧石片 x2, new 石矛 +2 x2) -> 38 cards, 24 weapons, 10 food
- Bram: 重击, rolls two attack dice and keeps the higher (was: ignore armor)
- Agatha: crafting makes a weapon only (no shield; a 'shield' request crafts a weapon)
- prompt table and rules doc no longer mention armor; the engine keeps armor as a
  card type so it can come back via the sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -636,7 +636,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>当前牌数(6 人局,共 42 张):外区每区 8 张,中心 10 张;食物共 10 张。张数填 0 = 暂时移出牌堆。</t>
+          <t>当前牌数(6 人局,共 38 张):林/水各 7 张,石/城各 8 张,中心 8 张;食物共 10 张;已无护甲。张数填 0 = 暂时移出牌堆。</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>合成(附加行动)：将两张初级武器合成——做成一把攻击=两者相加的武器，或一面减伤 2 的护盾。</t>
+          <t>合成(附加行动):将两张初级武器合成一把武器,攻击 = 两者相加。</t>
         </is>
       </c>
       <c r="G5" s="5" t="n"/>
@@ -1221,13 +1221,13 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>蛮力：攻击时无视对方护甲(护甲不减伤，也不被消耗)。</t>
+          <t>重击:攻击时掷两次骰子,取较高的一次。</t>
         </is>
       </c>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>进攻/克制防御流</t>
+          <t>进攻型;护甲移除后由"无视护甲"改为重击</t>
         </is>
       </c>
     </row>
@@ -1373,6 +1373,7 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1384,6 +1385,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -1720,11 +1722,11 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -1882,6 +1884,7 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -1893,6 +1896,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -2234,11 +2238,11 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -2396,6 +2400,7 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2407,6 +2412,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -2435,7 +2441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2558,9 +2564,13 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 护甲已从游戏中移除(2026-09)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2589,11 +2599,11 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -2624,11 +2634,11 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2669,7 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="5" t="n"/>
     </row>
@@ -2690,7 +2700,7 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
@@ -2769,15 +2779,39 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>石08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>武器</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>石矛</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>一根绑着尖石的木杆,戳人很疼</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Claude 补充(替换护甲)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -2922,26 +2956,39 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="25">
-      <c r="G25" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>张数合计</t>
         </is>
       </c>
-      <c r="H25" s="8">
-        <f>SUM(H3:H23)</f>
+      <c r="H26" s="8">
+        <f>SUM(H3:H25)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A27:F29"/>
@@ -3413,6 +3460,7 @@
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -3424,6 +3472,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
@@ -3929,11 +3978,11 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -3964,11 +4013,11 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Claude 补充</t>
+          <t>Claude 补充;张数 0 = 护甲已从游戏中移除(2026-09)</t>
         </is>
       </c>
     </row>
@@ -4126,6 +4175,7 @@
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -4137,6 +4187,7 @@
         <v/>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
@@ -4624,7 +4675,6 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4636,7 +4686,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -5107,7 +5156,6 @@
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -5119,7 +5167,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: city = 6 fragments + 2 food, forest/water get their 4th food back
Every zone now holds 8 cards: 40 in all (21 weapons, 13 food, 6 fragments).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -636,7 +636,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>当前牌数(6 人局,共 38 张):林/水各 7 张,石/城各 8 张,中心 8 张;食物共 10 张;已无护甲。张数填 0 = 暂时移出牌堆。</t>
+          <t>当前牌数(6 人局,共 40 张):每区 8 张;林/水 = 武器4+食物4,石 = 武器7+食物1,城 = 碎片6+食物2,中心 = 高级武器6+食物2;已无护甲。张数填 0 = 暂时移出牌堆。</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,6 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1385,7 +1384,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -1625,13 +1623,9 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2141,13 +2135,9 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2441,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2967,7 +2957,6 @@
       <c r="H24" s="6" t="n"/>
       <c r="I24" s="6" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="G26" s="7" t="inlineStr">
         <is>
@@ -2980,15 +2969,8 @@
       </c>
     </row>
     <row r="27"/>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>四个外区每区 8 张(数量一致);张数填 0 = 这张牌暂时不放进牌堆。外区只有初级武器(+1/+2);高级武器和特殊武器只在中心。类型用下拉菜单选:武器/食物/护甲/碎片。数值:武器=攻击加成,食物=回血,护甲=减伤,碎片=1。数值写成 +2Health、+2 防御 也能识别。张数 = 这张牌在本区牌堆里放几张。</t>
-        </is>
-      </c>
-    </row>
+    <row r="28"/>
     <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A27:F29"/>
@@ -3131,13 +3113,9 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>张数 0 = 暂时移出牌堆(2026-09 精简)</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -3232,9 +3210,13 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 城区只放碎片和食物(2026-09)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3263,9 +3245,13 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>张数 0 = 城区只放碎片和食物(2026-09)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -3298,7 +3284,7 @@
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
@@ -4175,7 +4161,6 @@
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -4187,7 +4172,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: two HP tiers, 10 and 12 (Fae, Iris, Michael 8 -> 10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Arena牌堆表.xlsx
+++ b/Arena牌堆表.xlsx
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>2</v>
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>2</v>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>3</v>
@@ -1373,6 +1373,7 @@
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1384,10 +1385,11 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP 量级 11/13/15、攻击 2/3/4,均为初值 🔧。</t>
+          <t>玩家 = 1 张人物牌 + 1 张隐藏身份牌。技能示例:『可攻击相邻区域』『一次抽多张物资』。HP 两档 10/12、攻击 2/3/4。</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1880,6 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -1890,7 +1891,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -2390,7 +2390,6 @@
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="G25" s="7" t="inlineStr">
         <is>
@@ -2402,7 +2401,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -3446,7 +3444,6 @@
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -3458,7 +3455,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>

</xml_diff>